<commit_message>
Day-22- Render the app titles in two columns
</commit_message>
<xml_diff>
--- a/Day wise tracker.xlsx
+++ b/Day wise tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/57b5ca6df9311485/Desktop/Udemy/Python Course/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="8_{A48CCA7A-F28D-4CEC-8D28-556C41702FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9912A2F2-48B2-4594-BF6C-D8FA2B8A0574}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="8_{A48CCA7A-F28D-4CEC-8D28-556C41702FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EC55FC3-E4EF-40FA-A625-6637366FD0BC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CDE4CE16-4524-4BED-9790-32B3A6313FC0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="100">
   <si>
     <t>Python Udemy Certification</t>
   </si>
@@ -335,16 +335,7 @@
     <t>C</t>
   </si>
   <si>
-    <t>4-7 July</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>Gaps in Between</t>
-  </si>
-  <si>
-    <t>DCET</t>
+    <t>Gaps in Between-DCET or Home or Weekend</t>
   </si>
 </sst>
 </file>
@@ -779,7 +770,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCA0B117-7917-4960-8EFD-7AC1B6A5469C}">
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.21875" customWidth="1"/>
@@ -787,11 +778,11 @@
     <col min="3" max="3" width="11.109375" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" customWidth="1"/>
-    <col min="9" max="9" width="22.109375" customWidth="1"/>
+    <col min="8" max="8" width="36.88671875" customWidth="1"/>
+    <col min="9" max="9" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -799,7 +790,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -816,7 +807,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -833,7 +824,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -850,7 +841,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -867,7 +858,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -884,7 +875,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -900,14 +891,8 @@
       <c r="E7" t="s">
         <v>98</v>
       </c>
-      <c r="H7" t="s">
-        <v>99</v>
-      </c>
-      <c r="I7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -924,13 +909,10 @@
         <v>98</v>
       </c>
       <c r="H8" t="s">
-        <v>101</v>
-      </c>
-      <c r="I8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -947,7 +929,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -964,7 +946,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -981,7 +963,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -998,7 +980,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1015,7 +997,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1032,7 +1014,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1049,7 +1031,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1193,7 +1175,7 @@
         <v>68</v>
       </c>
       <c r="C24" s="1">
-        <v>45861</v>
+        <v>45868</v>
       </c>
       <c r="D24" t="s">
         <v>69</v>
@@ -1207,7 +1189,7 @@
         <v>68</v>
       </c>
       <c r="C25" s="1">
-        <v>45862</v>
+        <v>45869</v>
       </c>
       <c r="D25" t="s">
         <v>69</v>
@@ -1221,7 +1203,7 @@
         <v>68</v>
       </c>
       <c r="C26" s="1">
-        <v>45863</v>
+        <v>45870</v>
       </c>
       <c r="D26" t="s">
         <v>70</v>
@@ -1235,7 +1217,7 @@
         <v>68</v>
       </c>
       <c r="C27" s="1">
-        <v>45866</v>
+        <v>45873</v>
       </c>
       <c r="D27" t="s">
         <v>71</v>
@@ -1249,7 +1231,7 @@
         <v>68</v>
       </c>
       <c r="C28" s="1">
-        <v>45867</v>
+        <v>45874</v>
       </c>
       <c r="D28" t="s">
         <v>71</v>
@@ -1263,7 +1245,7 @@
         <v>72</v>
       </c>
       <c r="C29" s="1">
-        <v>45868</v>
+        <v>45875</v>
       </c>
       <c r="D29" t="s">
         <v>73</v>
@@ -1277,7 +1259,7 @@
         <v>72</v>
       </c>
       <c r="C30" s="1">
-        <v>45869</v>
+        <v>45876</v>
       </c>
       <c r="D30" t="s">
         <v>73</v>
@@ -1291,7 +1273,7 @@
         <v>72</v>
       </c>
       <c r="C31" s="1">
-        <v>45870</v>
+        <v>45877</v>
       </c>
       <c r="D31" t="s">
         <v>74</v>
@@ -1305,7 +1287,7 @@
         <v>72</v>
       </c>
       <c r="C32" s="1">
-        <v>45873</v>
+        <v>45880</v>
       </c>
       <c r="D32" t="s">
         <v>74</v>
@@ -1319,7 +1301,7 @@
         <v>72</v>
       </c>
       <c r="C33" s="1">
-        <v>45874</v>
+        <v>45881</v>
       </c>
       <c r="D33" t="s">
         <v>74</v>
@@ -1333,7 +1315,7 @@
         <v>75</v>
       </c>
       <c r="C34" s="1">
-        <v>45875</v>
+        <v>45882</v>
       </c>
       <c r="D34" t="s">
         <v>76</v>
@@ -1347,7 +1329,7 @@
         <v>75</v>
       </c>
       <c r="C35" s="1">
-        <v>45876</v>
+        <v>45883</v>
       </c>
       <c r="D35" t="s">
         <v>76</v>
@@ -1361,7 +1343,7 @@
         <v>75</v>
       </c>
       <c r="C36" s="1">
-        <v>45877</v>
+        <v>45884</v>
       </c>
       <c r="D36" t="s">
         <v>77</v>
@@ -1375,7 +1357,7 @@
         <v>75</v>
       </c>
       <c r="C37" s="1">
-        <v>45880</v>
+        <v>45887</v>
       </c>
       <c r="D37" t="s">
         <v>77</v>
@@ -1389,7 +1371,7 @@
         <v>75</v>
       </c>
       <c r="C38" s="1">
-        <v>45881</v>
+        <v>45888</v>
       </c>
       <c r="D38" t="s">
         <v>78</v>
@@ -1403,7 +1385,7 @@
         <v>75</v>
       </c>
       <c r="C39" s="1">
-        <v>45882</v>
+        <v>45889</v>
       </c>
       <c r="D39" t="s">
         <v>78</v>
@@ -1417,7 +1399,7 @@
         <v>79</v>
       </c>
       <c r="C40" s="1">
-        <v>45883</v>
+        <v>45890</v>
       </c>
       <c r="D40" t="s">
         <v>80</v>
@@ -1431,7 +1413,7 @@
         <v>79</v>
       </c>
       <c r="C41" s="1">
-        <v>45884</v>
+        <v>45891</v>
       </c>
       <c r="D41" t="s">
         <v>80</v>
@@ -1445,7 +1427,7 @@
         <v>81</v>
       </c>
       <c r="C42" s="1">
-        <v>45887</v>
+        <v>45894</v>
       </c>
       <c r="D42" t="s">
         <v>83</v>
@@ -1459,7 +1441,7 @@
         <v>81</v>
       </c>
       <c r="C43" s="1">
-        <v>45888</v>
+        <v>45895</v>
       </c>
       <c r="D43" t="s">
         <v>84</v>
@@ -1473,7 +1455,7 @@
         <v>81</v>
       </c>
       <c r="C44" s="1">
-        <v>45889</v>
+        <v>45896</v>
       </c>
       <c r="D44" t="s">
         <v>84</v>
@@ -1487,7 +1469,7 @@
         <v>81</v>
       </c>
       <c r="C45" s="1">
-        <v>45890</v>
+        <v>45897</v>
       </c>
       <c r="D45" t="s">
         <v>84</v>
@@ -1501,7 +1483,7 @@
         <v>81</v>
       </c>
       <c r="C46" s="1">
-        <v>45891</v>
+        <v>45898</v>
       </c>
       <c r="D46" t="s">
         <v>82</v>
@@ -1515,7 +1497,7 @@
         <v>85</v>
       </c>
       <c r="C47" s="1">
-        <v>45894</v>
+        <v>45899</v>
       </c>
       <c r="D47" t="s">
         <v>91</v>
@@ -1529,7 +1511,7 @@
         <v>85</v>
       </c>
       <c r="C48" s="1">
-        <v>45895</v>
+        <v>45901</v>
       </c>
       <c r="D48" t="s">
         <v>91</v>
@@ -1543,7 +1525,7 @@
         <v>85</v>
       </c>
       <c r="C49" s="1">
-        <v>45896</v>
+        <v>45902</v>
       </c>
       <c r="D49" t="s">
         <v>91</v>
@@ -1557,7 +1539,7 @@
         <v>85</v>
       </c>
       <c r="C50" s="1">
-        <v>45897</v>
+        <v>45903</v>
       </c>
       <c r="D50" t="s">
         <v>92</v>
@@ -1571,7 +1553,7 @@
         <v>85</v>
       </c>
       <c r="C51" s="1">
-        <v>45898</v>
+        <v>45904</v>
       </c>
       <c r="D51" t="s">
         <v>93</v>
@@ -1585,7 +1567,7 @@
         <v>86</v>
       </c>
       <c r="C52" s="1">
-        <v>45899</v>
+        <v>45905</v>
       </c>
       <c r="D52" t="s">
         <v>94</v>
@@ -1599,7 +1581,7 @@
         <v>86</v>
       </c>
       <c r="C53" s="1">
-        <v>45901</v>
+        <v>45908</v>
       </c>
       <c r="D53" t="s">
         <v>94</v>
@@ -1613,7 +1595,7 @@
         <v>86</v>
       </c>
       <c r="C54" s="1">
-        <v>45902</v>
+        <v>45909</v>
       </c>
       <c r="D54" t="s">
         <v>95</v>
@@ -1627,7 +1609,7 @@
         <v>86</v>
       </c>
       <c r="C55" s="1">
-        <v>45903</v>
+        <v>45910</v>
       </c>
       <c r="D55" t="s">
         <v>95</v>
@@ -1641,7 +1623,7 @@
         <v>86</v>
       </c>
       <c r="C56" s="1">
-        <v>45904</v>
+        <v>45911</v>
       </c>
       <c r="D56" t="s">
         <v>95</v>
@@ -1655,7 +1637,7 @@
         <v>86</v>
       </c>
       <c r="C57" s="1">
-        <v>45905</v>
+        <v>45912</v>
       </c>
       <c r="D57" t="s">
         <v>96</v>
@@ -1669,7 +1651,7 @@
         <v>86</v>
       </c>
       <c r="C58" s="1">
-        <v>45908</v>
+        <v>45913</v>
       </c>
       <c r="D58" t="s">
         <v>96</v>
@@ -1683,7 +1665,7 @@
         <v>86</v>
       </c>
       <c r="C59" s="1">
-        <v>45909</v>
+        <v>45914</v>
       </c>
       <c r="D59" t="s">
         <v>96</v>
@@ -1697,7 +1679,7 @@
         <v>87</v>
       </c>
       <c r="C60" s="1">
-        <v>45910</v>
+        <v>45915</v>
       </c>
       <c r="D60" t="s">
         <v>89</v>
@@ -1711,7 +1693,7 @@
         <v>87</v>
       </c>
       <c r="C61" s="1">
-        <v>45911</v>
+        <v>45916</v>
       </c>
       <c r="D61" t="s">
         <v>89</v>
@@ -1725,7 +1707,7 @@
         <v>88</v>
       </c>
       <c r="C62" s="1">
-        <v>45912</v>
+        <v>45917</v>
       </c>
       <c r="D62" t="s">
         <v>90</v>

</xml_diff>